<commit_message>
feat(ecs): taskdef Role 이름 안정화 + admin UI PPTX 도형 정합 + xlsx 매핑
ecs/taskdef:
- admin/lifesync360 taskdef Role ARN: hash 박힌 이름 → lifesync-dev-EcsTaskExecutionRole / lifesync-dev-EcsTaskRole
  (21 yaml RoleName 명시와 매치)

admin UI:
- 5 → 4메뉴 (data_integrity 제거)
- dashboard PPTX slide1 도형 의도 — KPI 9 + 큰 박스 4 (AWS/GCP/S3/연령별가입률) + 최근 업로드 표
- customer 360 PPTX slide2 — 검색 단일 결과 + 메인 3 박스 + 하단 2 박스
- ai PPTX slide3 — 4컬럼×2행 그리드 + 보조 row
- ops PPTX slide4 — 네트워크 6 카드 + 백엔드 6 + 계열사 7 (3+4) + Wearable 6
- CSS 공백 최소화 (.card padding 22 → 8, .page-body padding 28 → 10)

docs:
- iac-handoff §7 — Role 이름 안정화 + secrets 권한 + Lambda Invoke + DynamoDB 권한
- 통합_문서1_매핑추가.xlsx — 15개 API 행 Backend 구현/엔드포인트/데이터소스 매핑 갱신

Co-Authored-By: Claude Opus 4.7 (1M context) <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/통합_문서1_매핑추가.xlsx
+++ b/통합_문서1_매핑추가.xlsx
@@ -1163,17 +1163,17 @@
       </c>
       <c r="C21" s="15" t="inlineStr">
         <is>
-          <t>AWS API Gateway → Lambda</t>
+          <t>admin-platform/app.py @app.route("/dashboard")  + boto3 ping</t>
         </is>
       </c>
       <c r="D21" s="15" t="inlineStr">
         <is>
-          <t>GET /api/dashboard/summary</t>
+          <t>GET /dashboard (관리자 페이지) · BFF Lambda 전환 시 GET /api/dashboard/summary</t>
         </is>
       </c>
       <c r="E21" s="15" t="inlineStr">
         <is>
-          <t>위 KPI 카드(3~11행) 집계 결과 통합 반환</t>
+          <t>집계: Aurora customer_recommend_history COUNT + DynamoDB lifesync_customer_result scan + customer_dashboard_log DISTINCT global_id</t>
         </is>
       </c>
     </row>
@@ -1190,17 +1190,17 @@
       </c>
       <c r="C22" s="15" t="inlineStr">
         <is>
-          <t>AWS API Gateway → Lambda</t>
+          <t>admin-platform/app.py _ping_s3_ingestion()  · boto3 s3 list_objects_v2</t>
         </is>
       </c>
       <c r="D22" s="15" t="inlineStr">
         <is>
-          <t>GET /api/s3/status</t>
+          <t>admin Flask 내부 호출 (운영 시 GET /api/s3/status)</t>
         </is>
       </c>
       <c r="E22" s="15" t="inlineStr">
         <is>
-          <t>S3 ListObjectsV2 + Inventory + EventBridge 기반 적재 상태</t>
+          <t>s3://lifesync-raw  ListObjectsV2 KeyCount + dt=YYYY-MM-DD 파티션 카운트 + EventBridge PutObject</t>
         </is>
       </c>
     </row>
@@ -1217,17 +1217,17 @@
       </c>
       <c r="C23" s="15" t="inlineStr">
         <is>
-          <t>AWS API Gateway → Lambda</t>
+          <t>admin-platform/app.py _ping_cloud_status()  · boto3 rds/dynamodb/elasticache/ecs/elbv2 describe-*</t>
         </is>
       </c>
       <c r="D23" s="15" t="inlineStr">
         <is>
-          <t>GET /api/cloud/status</t>
+          <t>admin Flask 내부 호출 (운영 시 GET /api/cloud/status)</t>
         </is>
       </c>
       <c r="E23" s="15" t="inlineStr">
         <is>
-          <t>CloudWatch Health + BigQuery Jobs API (AWS/GCP 통합 헬스)</t>
+          <t>AWS describe-db-clusters/list-tables/describe-cache-clusters/list-clusters + GCP stub (Vertex AI Model.list / BigQuery datasets.get)</t>
         </is>
       </c>
     </row>
@@ -1688,17 +1688,17 @@
       </c>
       <c r="C43" s="15" t="inlineStr">
         <is>
-          <t>AWS API GW → Lambda → Aurora + MySQL</t>
+          <t>admin-platform/app.py @app.route("/users/&lt;global_id&gt;") · _call_onprem("get_consent") + Aurora 직접 쿼리</t>
         </is>
       </c>
       <c r="D43" s="15" t="inlineStr">
         <is>
-          <t>GET /api/customer/profile/{global_id}</t>
+          <t>GET /users/&lt;global_id&gt;  →  내부 호출: PrivateAPI GET /internal/customer/{global_id} (TGW VPN 경유)</t>
         </is>
       </c>
       <c r="E43" s="15" t="inlineStr">
         <is>
-          <t>master_customer + users + customer_360_profile JOIN</t>
+          <t>On-Prem master_customer + customer_360_profile + users JOIN · DynamoDB lifesync_customer_result (점수/등급)</t>
         </is>
       </c>
     </row>
@@ -1715,17 +1715,17 @@
       </c>
       <c r="C44" s="15" t="inlineStr">
         <is>
-          <t>AWS API GW → Lambda → Redis</t>
+          <t>admin-platform/app.py _stub_redis_personalized()  (또는 lifesync360-platform/app.py /api/recommendations)</t>
         </is>
       </c>
       <c r="D44" s="15" t="inlineStr">
         <is>
-          <t>GET /api/customer/recommend/{global_id}</t>
+          <t>GET rec:{global_id} (Redis 직접) · cache miss 시 Aurora customer_recommend_history fallback</t>
         </is>
       </c>
       <c r="E44" s="15" t="inlineStr">
         <is>
-          <t>GET rec:{global_id}  (cache miss 시 Aurora fallback)</t>
+          <t>ElastiCache Redis ZREVRANGE rec:{global_id} 0 N WITHSCORES · TTL 6h</t>
         </is>
       </c>
     </row>
@@ -1742,17 +1742,17 @@
       </c>
       <c r="C45" s="15" t="inlineStr">
         <is>
-          <t>AWS API GW → Lambda → Aurora</t>
+          <t>admin-platform/app.py /users/&lt;gid&gt; 안에서 Aurora 직접 쿼리 (pymysql)</t>
         </is>
       </c>
       <c r="D45" s="15" t="inlineStr">
         <is>
-          <t>GET /api/customer/history/{global_id}</t>
+          <t>admin Flask 내부 호출 (운영 시 GET /api/customer/history/{id})</t>
         </is>
       </c>
       <c r="E45" s="15" t="inlineStr">
         <is>
-          <t>customer_recommend_history WHERE global_id=?</t>
+          <t>Aurora customer_recommend_history WHERE global_id=? ORDER BY recommended_at DESC LIMIT N</t>
         </is>
       </c>
     </row>
@@ -1769,17 +1769,17 @@
       </c>
       <c r="C46" s="15" t="inlineStr">
         <is>
-          <t>AWS API GW → Lambda → Aurora</t>
+          <t>admin-platform/app.py (Aurora customer_dashboard_log 직접)</t>
         </is>
       </c>
       <c r="D46" s="15" t="inlineStr">
         <is>
-          <t>GET /api/customer/activity/{global_id}</t>
+          <t>admin Flask 내부 호출 (운영 시 GET /api/customer/activity/{id})</t>
         </is>
       </c>
       <c r="E46" s="15" t="inlineStr">
         <is>
-          <t>customer_dashboard_log WHERE global_id=?</t>
+          <t>Aurora customer_dashboard_log WHERE global_id=? ORDER BY view_time DESC</t>
         </is>
       </c>
     </row>
@@ -2298,17 +2298,17 @@
       </c>
       <c r="C69" s="15" t="inlineStr">
         <is>
-          <t>AWS API GW → Lambda → BigQuery</t>
+          <t>admin-platform/app.py @app.route("/ai") · Aurora 직접 GROUP BY (현재 구현, BigQuery 미연동)</t>
         </is>
       </c>
       <c r="D69" s="15" t="inlineStr">
         <is>
-          <t>GET /api/ai/recommend-stats</t>
+          <t>GET /ai (관리자 페이지) · BigQuery 연동 시 GET /api/ai/recommend-stats</t>
         </is>
       </c>
       <c r="E69" s="15" t="inlineStr">
         <is>
-          <t>lifesync_curated.recommendation_mart 집계 (CTR/CVR/Top10)</t>
+          <t>Aurora customer_recommend_history GROUP BY product/category. 운영 시 BQ lifesync_curated.recommendation_mart 로 대체</t>
         </is>
       </c>
     </row>
@@ -2325,17 +2325,17 @@
       </c>
       <c r="C70" s="15" t="inlineStr">
         <is>
-          <t>AWS API GW → Lambda → BigQuery (PSC Endpoint)</t>
+          <t>(현재 미구현 — mockup_data.py · MOCKUP_RECOMMEND_TREND/BY_CATEGORY/BY_GRADE)</t>
         </is>
       </c>
       <c r="D70" s="15" t="inlineStr">
         <is>
-          <t>GET /api/bigquery/analytics</t>
+          <t>운영 시 GET /api/bigquery/analytics → Lambda (PSC Endpoint) → BigQuery</t>
         </is>
       </c>
       <c r="E70" s="15" t="inlineStr">
         <is>
-          <t>lifesync_serving.* View 호출 (v_user_dashboard 등)</t>
+          <t>BQ lifesync_curated.recommendation_mart + lifesync_serving.v_vip_customer + score_mart</t>
         </is>
       </c>
     </row>
@@ -2352,17 +2352,17 @@
       </c>
       <c r="C71" s="15" t="inlineStr">
         <is>
-          <t>AWS API GW → Lambda → Vertex AI API</t>
+          <t>(현재 미구현 — mockup_data.py · MOCKUP_VERTEX_AI / MOCKUP_FEATURE_IMPORTANCE)</t>
         </is>
       </c>
       <c r="D71" s="15" t="inlineStr">
         <is>
-          <t>GET /api/vertex/metrics</t>
+          <t>운영 시 GET /api/vertex/metrics → Lambda → Vertex AI API</t>
         </is>
       </c>
       <c r="E71" s="15" t="inlineStr">
         <is>
-          <t>Vertex AI Model.evaluations.get — accuracy/precision/recall</t>
+          <t>Vertex AI Model.evaluations.get  (auc/accuracy/precision/recall) + GCS feature_importance.json</t>
         </is>
       </c>
     </row>
@@ -3074,17 +3074,17 @@
       </c>
       <c r="C102" s="15" t="inlineStr">
         <is>
-          <t>AWS API GW → Lambda → CloudWatch</t>
+          <t>admin-platform/app.py _ping_tgw()  · boto3 ec2 describe-transit-gateways/-attachments</t>
         </is>
       </c>
       <c r="D102" s="15" t="inlineStr">
         <is>
-          <t>GET /api/network/tgw</t>
+          <t>admin Flask 내부 호출 (운영 시 GET /api/network/tgw)</t>
         </is>
       </c>
       <c r="E102" s="15" t="inlineStr">
         <is>
-          <t>TGW 메트릭 (BytesIn/Out, Attachment 상태)</t>
+          <t>AWS EC2 describe-transit-gateways · CloudWatch TGW BytesIn/Out</t>
         </is>
       </c>
     </row>
@@ -3101,17 +3101,17 @@
       </c>
       <c r="C103" s="15" t="inlineStr">
         <is>
-          <t>AWS API GW → Lambda → CloudWatch</t>
+          <t>admin-platform/app.py _ping_vpn()  · boto3 ec2 describe-vpn-connections</t>
         </is>
       </c>
       <c r="D103" s="15" t="inlineStr">
         <is>
-          <t>GET /api/network/vpn</t>
+          <t>admin Flask 내부 호출 (운영 시 GET /api/network/vpn)</t>
         </is>
       </c>
       <c r="E103" s="15" t="inlineStr">
         <is>
-          <t>VPN TunnelState / DataIn / DataOut</t>
+          <t>AWS EC2 describe-vpn-connections.Tunnels · CloudWatch TunnelState/TunnelDataIn-Out</t>
         </is>
       </c>
     </row>
@@ -3128,17 +3128,17 @@
       </c>
       <c r="C104" s="15" t="inlineStr">
         <is>
-          <t>AWS API GW → Lambda → EC2 API + CloudWatch</t>
+          <t>admin-platform/app.py _ping_vm_status()  · boto3 ec2 describe-instances (tag:Project=lifesync)</t>
         </is>
       </c>
       <c r="D104" s="15" t="inlineStr">
         <is>
-          <t>GET /api/vm/group</t>
+          <t>admin Flask 내부 호출 (운영 시 GET /api/vm/group)</t>
         </is>
       </c>
       <c r="E104" s="15" t="inlineStr">
         <is>
-          <t>Group VM (VPC) EC2 인스턴스 상태 + CPU/MEM</t>
+          <t>AWS EC2 describe-instances State + CloudWatch CPUUtilization/mem_used_percent (CW Agent)</t>
         </is>
       </c>
     </row>
@@ -3155,17 +3155,17 @@
       </c>
       <c r="C105" s="15" t="inlineStr">
         <is>
-          <t>AWS API GW → Lambda → Kinesis + CloudWatch</t>
+          <t>admin-platform/app.py _ping_wearable_realtime()  · boto3 cloudwatch get-metric-statistics</t>
         </is>
       </c>
       <c r="D105" s="15" t="inlineStr">
         <is>
-          <t>GET /api/vm/wearable</t>
+          <t>admin Flask 내부 호출 (운영 시 GET /api/vm/wearable)</t>
         </is>
       </c>
       <c r="E105" s="15" t="inlineStr">
         <is>
-          <t>Kinesis IncomingRecords + Wearable EC2 헬스</t>
+          <t>CloudWatch custom namespace LifeSync/Wearable · heart_rate / blood_pressure / spo2 / steps / alerts / send_rate</t>
         </is>
       </c>
     </row>
@@ -3182,17 +3182,17 @@
       </c>
       <c r="C106" s="15" t="inlineStr">
         <is>
-          <t>On-Prem private API → VPN</t>
+          <t>admin-platform/app.py _ping_local_lab()  · _call_onprem("local_lab_status")  via TGW VPN</t>
         </is>
       </c>
       <c r="D106" s="15" t="inlineStr">
         <is>
-          <t>GET /api/local/status</t>
+          <t>admin Flask 내부 호출 → Lambda onprem-query-lambda → PrivateAPI (192.168.56.13)</t>
         </is>
       </c>
       <c r="E106" s="15" t="inlineStr">
         <is>
-          <t>ls-db / ls-token VM 상태 (192.168.56.0/24)</t>
+          <t>On-Prem VirtualBox VM 상태 (ls-vpngw/ls-db/ls-token/ls-api) · systemd / docker ps</t>
         </is>
       </c>
     </row>

</xml_diff>